<commit_message>
Finished Full Analysis for Pipeline scenario
</commit_message>
<xml_diff>
--- a/Pipeline/OverallStatsPipeline-noboot.xlsx
+++ b/Pipeline/OverallStatsPipeline-noboot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexb\OneDrive\Documents\Thesis\Pipeline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3687AD36-2890-45E3-A6FF-F6BAD97D16E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11CB8E1D-A373-4E27-8580-E1ED96F2178F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{10219E88-FFE1-4721-B87F-58FBE8BDB343}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{10219E88-FFE1-4721-B87F-58FBE8BDB343}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
   <si>
     <t>Program</t>
   </si>
@@ -129,6 +129,30 @@
   </si>
   <si>
     <t>Nu: 0.2, Gamma: 0.7</t>
+  </si>
+  <si>
+    <t>Nu: 0.5, Gamma: 0.2</t>
+  </si>
+  <si>
+    <t>Nu: 0.9, Gamma: 0.9</t>
+  </si>
+  <si>
+    <t>Nu: 0.99, Gamma: 0.0002</t>
+  </si>
+  <si>
+    <t>Nu: 0.9, Gamma: 0.5</t>
+  </si>
+  <si>
+    <t>Nu: 0.2, Gamma: 0.9</t>
+  </si>
+  <si>
+    <t>Nu: 0.5, Gamma: 0.7</t>
+  </si>
+  <si>
+    <t>Nu: 0.99, Gamma: 0.99</t>
+  </si>
+  <si>
+    <t>Nu: 0.5, Gamma: 0.99</t>
   </si>
 </sst>
 </file>
@@ -501,19 +525,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{263ED5F6-01AE-4A3B-A6DC-B2A5E21A756E}">
   <dimension ref="A1:M15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" customWidth="1"/>
-    <col min="2" max="2" width="21.26953125" customWidth="1"/>
-    <col min="12" max="12" width="12.26953125" customWidth="1"/>
+    <col min="1" max="1" width="19.77734375" customWidth="1"/>
+    <col min="2" max="2" width="21.21875" customWidth="1"/>
+    <col min="12" max="12" width="12.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -524,10 +548,10 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
         <v>3</v>
-      </c>
-      <c r="E2" t="s">
-        <v>4</v>
       </c>
       <c r="F2" t="s">
         <v>5</v>
@@ -554,7 +578,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -577,12 +601,12 @@
         <v>93.75</v>
       </c>
       <c r="H3">
-        <f>(C3)/(C3+D3)</f>
-        <v>1</v>
+        <f>(C3)/(C3+E3)</f>
+        <v>0.66666666666666663</v>
       </c>
       <c r="I3">
-        <f>C3/(C3+E3)</f>
-        <v>0.66666666666666663</v>
+        <f>C3/(C3+D3)</f>
+        <v>1</v>
       </c>
       <c r="J3">
         <f>(2*(H3*I3))/(H3+I3)</f>
@@ -599,7 +623,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -621,20 +645,20 @@
       <c r="G4">
         <v>91.1111111111111</v>
       </c>
-      <c r="H4">
-        <f t="shared" ref="H4:H12" si="0">(C4)/(C4+D4)</f>
-        <v>0</v>
-      </c>
-      <c r="I4" t="e">
-        <f t="shared" ref="I4:I13" si="1">C4/(C4+E4)</f>
+      <c r="H4" t="e">
+        <f t="shared" ref="H4:H15" si="0">(C4)/(C4+E4)</f>
         <v>#DIV/0!</v>
+      </c>
+      <c r="I4">
+        <f t="shared" ref="I4:I15" si="1">C4/(C4+D4)</f>
+        <v>0</v>
       </c>
       <c r="J4" t="e">
         <f t="shared" ref="J4:J13" si="2">(2*(H4*I4))/(H4+I4)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="K4">
-        <f t="shared" ref="K4:K13" si="3">F4/(F4+D4)</f>
+        <f>F4/(F4+D4)</f>
         <v>0.91111111111111109</v>
       </c>
       <c r="L4">
@@ -644,7 +668,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -668,18 +692,18 @@
       </c>
       <c r="H5">
         <f t="shared" si="0"/>
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I5">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="J5">
         <f t="shared" si="2"/>
         <v>0.33333333333333337</v>
       </c>
       <c r="K5">
-        <f t="shared" si="3"/>
+        <f>F5/(F5+D5)</f>
         <v>0.92982456140350878</v>
       </c>
       <c r="L5">
@@ -689,7 +713,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -713,18 +737,18 @@
       </c>
       <c r="H6">
         <f t="shared" si="0"/>
-        <v>0.7</v>
+        <v>0.875</v>
       </c>
       <c r="I6">
         <f t="shared" si="1"/>
-        <v>0.875</v>
+        <v>0.7</v>
       </c>
       <c r="J6">
         <f t="shared" si="2"/>
         <v>0.77777777777777768</v>
       </c>
       <c r="K6">
-        <f t="shared" si="3"/>
+        <f>F6/(F6+D6)</f>
         <v>0.99986992715920919</v>
       </c>
       <c r="L6">
@@ -734,25 +758,43 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="H7" t="e">
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7">
+        <v>14</v>
+      </c>
+      <c r="D7">
+        <v>9</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>1268</v>
+      </c>
+      <c r="G7">
+        <v>99.302865995352406</v>
+      </c>
+      <c r="H7">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I7" t="e">
+        <v>1</v>
+      </c>
+      <c r="I7">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J7" t="e">
+        <v>0.60869565217391308</v>
+      </c>
+      <c r="J7">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K7" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>0.7567567567567568</v>
+      </c>
+      <c r="K7">
+        <f>F7/(F7+D7)</f>
+        <v>0.99295223179326542</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -761,25 +803,43 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="H8" t="e">
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>122</v>
+      </c>
+      <c r="G8">
+        <v>97.619047619047606</v>
+      </c>
+      <c r="H8">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I8" t="e">
+        <v>1</v>
+      </c>
+      <c r="I8">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J8" t="e">
+        <v>0.25</v>
+      </c>
+      <c r="J8">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K8" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>0.4</v>
+      </c>
+      <c r="K8">
+        <f>F8/(F8+D8)</f>
+        <v>0.97599999999999998</v>
       </c>
       <c r="L8">
         <v>0</v>
@@ -788,25 +848,43 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>15</v>
       </c>
-      <c r="H9" t="e">
+      <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>34</v>
+      </c>
+      <c r="G9">
+        <v>92.105263157894697</v>
+      </c>
+      <c r="H9">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I9" t="e">
-        <f>C9/(C9+E9)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J9" t="e">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="1"/>
+        <v>0.25</v>
+      </c>
+      <c r="J9">
         <f>(2*(H9*I9))/(H9+I9)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K9" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>0.4</v>
+      </c>
+      <c r="K9">
+        <f>F9/(F9+D9)</f>
+        <v>0.91891891891891897</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -815,25 +893,43 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>17</v>
       </c>
-      <c r="H10" t="e">
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>182</v>
+      </c>
+      <c r="G10">
+        <v>98.387096769999999</v>
+      </c>
+      <c r="H10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I10" t="e">
+        <v>1</v>
+      </c>
+      <c r="I10">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J10" t="e">
+        <v>0.25</v>
+      </c>
+      <c r="J10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K10" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>0.4</v>
+      </c>
+      <c r="K10">
+        <f>F10/(F10+D10)</f>
+        <v>0.98378378378378384</v>
       </c>
       <c r="L10">
         <v>0</v>
@@ -842,106 +938,178 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>26</v>
+      </c>
+      <c r="G11">
+        <v>86.6666666666666</v>
       </c>
       <c r="H11" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="I11" t="e">
+      <c r="I11">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="J11" t="e">
         <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="K11" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+      <c r="K11">
+        <f>F12/(F12+D12)</f>
+        <v>1</v>
       </c>
       <c r="L11">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M11">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
-      <c r="H12" t="e">
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12">
+        <v>12</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>291</v>
+      </c>
+      <c r="G12">
+        <v>99.671052631578902</v>
+      </c>
+      <c r="H12">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I12" t="e">
+        <v>0.92307692307692313</v>
+      </c>
+      <c r="I12">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J12" t="e">
+        <v>1</v>
+      </c>
+      <c r="J12">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0.96000000000000008</v>
       </c>
       <c r="K12" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <f>#REF!/(#REF!+#REF!)</f>
+        <v>#REF!</v>
       </c>
       <c r="L12">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M12">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>20</v>
       </c>
-      <c r="H13" t="e">
-        <f>(C13)/(C13+D13)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I13" t="e">
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>28</v>
+      </c>
+      <c r="G13">
+        <v>93.939393939393895</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I13">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J13" t="e">
+        <v>0.6</v>
+      </c>
+      <c r="J13">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K13" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>0.74999999999999989</v>
+      </c>
+      <c r="K13">
+        <f>F13/(F13+D13)</f>
+        <v>0.93333333333333335</v>
       </c>
       <c r="L13">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M13">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>21</v>
       </c>
-      <c r="H14" t="e">
-        <f t="shared" ref="H14:H15" si="4">(C14)/(C14+D14)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I14" t="e">
-        <f t="shared" ref="I14:I15" si="5">C14/(C14+E14)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J14" t="e">
-        <f t="shared" ref="J14:J15" si="6">(2*(H14*I14))/(H14+I14)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K14" t="e">
-        <f t="shared" ref="K14:K15" si="7">F14/(F14+D14)</f>
-        <v>#DIV/0!</v>
+      <c r="B14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>11</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>118</v>
+      </c>
+      <c r="G14">
+        <v>91.53846154</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="1"/>
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="J14">
+        <f t="shared" ref="J14:J15" si="3">(2*(H14*I14))/(H14+I14)</f>
+        <v>0.15384615384615385</v>
+      </c>
+      <c r="K14">
+        <f>F14/(F14+D14)</f>
+        <v>0.9147286821705426</v>
       </c>
       <c r="L14">
         <v>0</v>
@@ -950,25 +1118,43 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>22</v>
       </c>
-      <c r="H15" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I15" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J15" t="e">
-        <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K15" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15">
+        <v>251</v>
+      </c>
+      <c r="D15">
+        <v>251</v>
+      </c>
+      <c r="E15">
+        <v>77</v>
+      </c>
+      <c r="F15">
+        <v>4939</v>
+      </c>
+      <c r="G15">
+        <v>94.0558173251178</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="0"/>
+        <v>0.7652439024390244</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="3"/>
+        <v>0.60481927710843375</v>
+      </c>
+      <c r="K15">
+        <f>F15/(F15+D15)</f>
+        <v>0.95163776493256258</v>
       </c>
       <c r="L15">
         <v>0</v>

</xml_diff>